<commit_message>
Minor fix - Consolidated accuracy report
</commit_message>
<xml_diff>
--- a/evaluations/pv_consolidated_accuracy.xlsx
+++ b/evaluations/pv_consolidated_accuracy.xlsx
@@ -519,7 +519,7 @@
     <pageSetUpPr/>
   </sheetPr>
   <dimension ref="A1:AG301"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15" outlineLevelCol="0"/>
   <cols>
     <col width="8" customWidth="1" min="1" max="1"/>
     <col width="25" customWidth="1" min="2" max="2"/>
@@ -40658,8 +40658,8 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E43"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <dimension ref="A1:E44"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15" outlineLevelCol="0"/>
   <cols>
     <col width="48" customWidth="1" min="1" max="1"/>
     <col width="22" customWidth="1" min="2" max="2"/>
@@ -41166,22 +41166,34 @@
     <row r="42">
       <c r="A42" s="13" t="inlineStr">
         <is>
-          <t>Average Clinical Accuracy Score (out of 5.0)</t>
+          <t>LLM Judge Clinical Acceptability Rate (Score &gt;= 3)</t>
         </is>
       </c>
       <c r="B42" s="22" t="inlineStr">
         <is>
-          <t>4.28 / 5.0</t>
+          <t>93.3%</t>
         </is>
       </c>
     </row>
     <row r="43">
       <c r="A43" s="13" t="inlineStr">
         <is>
+          <t>Average Clinical Accuracy Score (out of 5.0)</t>
+        </is>
+      </c>
+      <c r="B43" s="22" t="inlineStr">
+        <is>
+          <t>4.28 / 5.0</t>
+        </is>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" s="13" t="inlineStr">
+        <is>
           <t>Inter-Method Agreement Rate</t>
         </is>
       </c>
-      <c r="B43" s="21" t="inlineStr">
+      <c r="B44" s="21" t="inlineStr">
         <is>
           <t>52.7%</t>
         </is>

</xml_diff>